<commit_message>
ScreenShots inListeners is implemented
</commit_message>
<xml_diff>
--- a/src/main/java/testData/TutorialNinjaTestData.xlsx
+++ b/src/main/java/testData/TutorialNinjaTestData.xlsx
@@ -28,7 +28,7 @@
     <t xml:space="preserve">Password</t>
   </si>
   <si>
-    <t xml:space="preserve">amotooricap9@gmail.com</t>
+    <t xml:space="preserve">amotooricap7@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">amotooricap3@gmail.com</t>
@@ -161,7 +161,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -171,6 +171,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -226,29 +230,29 @@
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="0" t="n">
         <v>12345</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="5" t="n">
         <v>12345</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>12345</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="amotooricap9@gmail.com"/>
+    <hyperlink ref="A2" r:id="rId1" display="amotooricap7@gmail.com"/>
     <hyperlink ref="A3" r:id="rId2" display="amotooricap3@gmail.com"/>
     <hyperlink ref="A4" r:id="rId3" display="amotooricap1@gmail.com"/>
   </hyperlinks>

</xml_diff>